<commit_message>
feat: change regex healthConditionOfInterest
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-checksum.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-checksum.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-26 16:19:40</t>
+          <t>2026-10-27 15:44:14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1798,7 +1798,11 @@
           <t>sh:Literal</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>xsd:hexBinary</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: fixes regex healthCondition, fixes dash Table.url, fixes Validationshapes
</commit_message>
<xml_diff>
--- a/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-checksum.xlsx
+++ b/Formalisation(shacl)/Core/SHACL_pipeline_templates/SHACL-checksum.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27 15:44:14</t>
+          <t>2026-10-28 09:50:43</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1798,11 +1798,7 @@
           <t>sh:Literal</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>xsd:hexBinary</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>

</xml_diff>